<commit_message>
PAUSED (task169): stage 4 round 1 fixes, waiting on round 2 readers
The call is the 2027 cohort's two-year return rate alone (20 per cent); the districts left the call because a
route without the decisive step ranked them right. The asks are re-sited onto grain devices on the readers' own
paths: one recommitment per parolee per hearing, the union of a parolee's overlapping detainers by half of 2025,
and writ trips ended by a release, with the rescission fork closed as not rescinded by 30 June 2026. The judge's
two near-miss readings are fork rows SF11 and SF12, both taking the decisive step.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task169/golden/returns_projection_2027.xlsx
+++ b/task169/golden/returns_projection_2027.xlsx
@@ -10,13 +10,14 @@
     <sheet name="Projection 2027" sheetId="1" r:id="rId1"/>
     <sheet name="Board revocations FY26" sheetId="2" r:id="rId2"/>
     <sheet name="Detainer days 2025" sheetId="3" r:id="rId3"/>
+    <sheet name="Writ days 2025" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
   <si>
     <t>Two-year returns of the 2027 parole releases under Act 26-114</t>
   </si>
@@ -27,48 +28,42 @@
     <t>Two-year return rate carried in the projection</t>
   </si>
   <si>
-    <t>District with the highest rate</t>
+    <t>Parole district</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
+  <si>
+    <t>2027 releases to parole</t>
+  </si>
+  <si>
+    <t>Estimated two-year return rate</t>
+  </si>
+  <si>
+    <t>Expected returns</t>
   </si>
   <si>
     <t>Garrison</t>
   </si>
   <si>
-    <t>District with the lowest rate</t>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>Ridgway</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>Linwood</t>
+  </si>
+  <si>
+    <t>D3</t>
   </si>
   <si>
     <t>Corliss</t>
   </si>
   <si>
-    <t>Parole district</t>
-  </si>
-  <si>
-    <t>Office</t>
-  </si>
-  <si>
-    <t>2027 releases to parole</t>
-  </si>
-  <si>
-    <t>Estimated two-year return rate</t>
-  </si>
-  <si>
-    <t>Expected returns</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>Ridgway</t>
-  </si>
-  <si>
-    <t>D2</t>
-  </si>
-  <si>
-    <t>Linwood</t>
-  </si>
-  <si>
-    <t>D3</t>
-  </si>
-  <si>
     <t>D4</t>
   </si>
   <si>
@@ -87,13 +82,13 @@
     <t>Each arrest's chance of a Department sentence and the time from arrest to admission are the courts' own, by charge grade (felony A-B, felony C-E, misdemeanour), from arrests to 30 June 2024 that went to court; arrests the Board answered by revoking parole are left out because no court decided them.</t>
   </si>
   <si>
-    <t>The rate is carried in steps of five percentage points (methodology 3.3); the district rates are shown at the model's precision for ranking only.</t>
-  </si>
-  <si>
-    <t>Parole revocations the Board ordered, 1 July 2025 to 30 June 2026, not rescinded</t>
-  </si>
-  <si>
-    <t>Legacy system actions to 2 January 2026 and the new case system from 5 January; entries the legacy system took for carried-over cases after its close are counted once, from the new system.</t>
+    <t>The rate is carried in steps of five percentage points (methodology 3.3); the district rates are the model's own, shown for the projection's district tables.</t>
+  </si>
+  <si>
+    <t>Recommitments the Board ordered, 1 July 2025 to 30 June 2026, not rescinded by 30 June 2026</t>
+  </si>
+  <si>
+    <t>One recommitment per parolee per hearing: two reports taken up at one hearing are one order. Legacy system to 2 January 2026, new case system from 5 January.</t>
   </si>
   <si>
     <t>District office</t>
@@ -111,25 +106,43 @@
     <t>All offices</t>
   </si>
   <si>
-    <t>Days parolees were held on Board detainers in each district's county jails, 2025</t>
-  </si>
-  <si>
-    <t>Counting the day a detainer was lodged and not the day the person left. A legacy detainer with no lift date ended when the person was admitted to the Department.</t>
-  </si>
-  <si>
-    <t>Jan-Mar 2025</t>
-  </si>
-  <si>
-    <t>Apr-Jun 2025</t>
-  </si>
-  <si>
-    <t>Jul-Sep 2025</t>
-  </si>
-  <si>
-    <t>Oct-Dec 2025</t>
+    <t>Parolee-days held on Board detainers in each district's county jails, 2025</t>
+  </si>
+  <si>
+    <t>A parolee held on two detainers at once is held once. Counting the day a detainer was lodged and not the day the person left; a legacy detainer with no lift date ended at the person's admission.</t>
+  </si>
+  <si>
+    <t>January to June</t>
+  </si>
+  <si>
+    <t>July to December</t>
   </si>
   <si>
     <t>Year</t>
+  </si>
+  <si>
+    <t>Days people spent out of each institution on court writs, 2025</t>
+  </si>
+  <si>
+    <t>Counting the day a person went out and not the day the trip ended. A trip ends at the return (WRI) or, for a person the court released, at the release.</t>
+  </si>
+  <si>
+    <t>Institution</t>
+  </si>
+  <si>
+    <t>SCI-KTR</t>
+  </si>
+  <si>
+    <t>SCI-FNW</t>
+  </si>
+  <si>
+    <t>SCI-DNM</t>
+  </si>
+  <si>
+    <t>SCI-LKV</t>
+  </si>
+  <si>
+    <t>SCI-BRW</t>
   </si>
 </sst>
 </file>
@@ -565,45 +578,29 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
     <row r="8" spans="1:5">
       <c r="A8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C9" s="6">
         <v>2385</v>
@@ -617,10 +614,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C10" s="6">
         <v>1713</v>
@@ -634,10 +631,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C11" s="6">
         <v>1385</v>
@@ -651,10 +648,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C12" s="6">
         <v>983</v>
@@ -668,7 +665,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C13" s="8">
         <v>6466</v>
@@ -682,27 +679,27 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -721,106 +718,106 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C5" s="6">
         <v>1586</v>
       </c>
       <c r="D5" s="6">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E5" s="6">
         <f>C5+D5</f>
-        <v>1881</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C6" s="6">
         <v>709</v>
       </c>
       <c r="D6" s="6">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E6" s="6">
         <f>C6+D6</f>
-        <v>968</v>
+        <v>971</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C7" s="6">
         <v>427</v>
       </c>
       <c r="D7" s="6">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E7" s="6">
         <f>C7+D7</f>
-        <v>603</v>
+        <v>606</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C8" s="6">
         <v>157</v>
       </c>
       <c r="D8" s="6">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E8" s="6">
         <f>C8+D8</f>
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" s="8">
         <f>SUM(C5:C8)</f>
@@ -828,11 +825,11 @@
       </c>
       <c r="D9" s="8">
         <f>SUM(D5:D8)</f>
-        <v>867</v>
+        <v>876</v>
       </c>
       <c r="E9" s="8">
         <f>SUM(E5:E8)</f>
-        <v>3746</v>
+        <v>3755</v>
       </c>
     </row>
   </sheetData>
@@ -842,125 +839,208 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="6" width="13.7109375" customWidth="1"/>
+    <col min="2" max="4" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="C4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="6">
+        <v>44780</v>
+      </c>
+      <c r="C5" s="6">
+        <v>49489</v>
+      </c>
+      <c r="D5" s="6">
+        <f>SUM(B5:C5)</f>
+        <v>94269</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="6">
+        <v>30248</v>
+      </c>
+      <c r="C6" s="6">
+        <v>27668</v>
+      </c>
+      <c r="D6" s="6">
+        <f>SUM(B6:C6)</f>
+        <v>57916</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="6">
+        <v>19991</v>
+      </c>
+      <c r="C7" s="6">
+        <v>21769</v>
+      </c>
+      <c r="D7" s="6">
+        <f>SUM(B7:C7)</f>
+        <v>41760</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="6">
+        <v>12729</v>
+      </c>
+      <c r="C8" s="6">
+        <v>12505</v>
+      </c>
+      <c r="D8" s="6">
+        <f>SUM(B8:C8)</f>
+        <v>25234</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="4" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" s="5" t="s">
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
       <c r="B5" s="6">
-        <v>22746</v>
+        <v>3736</v>
       </c>
       <c r="C5" s="6">
-        <v>22034</v>
+        <v>3929</v>
       </c>
       <c r="D5" s="6">
-        <v>24883</v>
-      </c>
-      <c r="E5" s="6">
-        <v>24606</v>
-      </c>
-      <c r="F5" s="6">
-        <f>SUM(B5:E5)</f>
-        <v>94269</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <f>SUM(B5:C5)</f>
+        <v>7665</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="B6" s="6">
-        <v>15421</v>
+        <v>3790</v>
       </c>
       <c r="C6" s="6">
-        <v>14827</v>
+        <v>3876</v>
       </c>
       <c r="D6" s="6">
-        <v>13663</v>
-      </c>
-      <c r="E6" s="6">
-        <v>14005</v>
-      </c>
-      <c r="F6" s="6">
-        <f>SUM(B6:E6)</f>
-        <v>57916</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <f>SUM(B6:C6)</f>
+        <v>7666</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="B7" s="6">
-        <v>9962</v>
+        <v>3657</v>
       </c>
       <c r="C7" s="6">
-        <v>10029</v>
+        <v>3574</v>
       </c>
       <c r="D7" s="6">
-        <v>10630</v>
-      </c>
-      <c r="E7" s="6">
-        <v>11139</v>
-      </c>
-      <c r="F7" s="6">
-        <f>SUM(B7:E7)</f>
-        <v>41760</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <f>SUM(B7:C7)</f>
+        <v>7231</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="B8" s="6">
-        <v>6338</v>
+        <v>3538</v>
       </c>
       <c r="C8" s="6">
-        <v>6391</v>
+        <v>4054</v>
       </c>
       <c r="D8" s="6">
-        <v>6354</v>
-      </c>
-      <c r="E8" s="6">
-        <v>6151</v>
-      </c>
-      <c r="F8" s="6">
-        <f>SUM(B8:E8)</f>
-        <v>25234</v>
+        <f>SUM(B8:C8)</f>
+        <v>7592</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="6">
+        <v>3595</v>
+      </c>
+      <c r="C9" s="6">
+        <v>4077</v>
+      </c>
+      <c r="D9" s="6">
+        <f>SUM(B9:C9)</f>
+        <v>7672</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PAUSED (task169): stage 4 round 2 fix, waiting on the re-judge
Writ movements are generated one trip at a time per person: two admissions with no release between them had
written overlapping writ loops, so no reading of the files reproduced Table 3. Every WRI now closes the one open
trip, next-WRI and same-institution pairing both give the golden, and no pairing or trip-end rule is filed. The
call, Tables 1 and 2 and every target file but the admissions table and its manifest row are byte-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task169/golden/returns_projection_2027.xlsx
+++ b/task169/golden/returns_projection_2027.xlsx
@@ -973,14 +973,14 @@
         <v>37</v>
       </c>
       <c r="B5" s="6">
-        <v>3736</v>
+        <v>3524</v>
       </c>
       <c r="C5" s="6">
-        <v>3929</v>
+        <v>3857</v>
       </c>
       <c r="D5" s="6">
         <f>SUM(B5:C5)</f>
-        <v>7665</v>
+        <v>7381</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -988,14 +988,14 @@
         <v>38</v>
       </c>
       <c r="B6" s="6">
-        <v>3790</v>
+        <v>3642</v>
       </c>
       <c r="C6" s="6">
-        <v>3876</v>
+        <v>3754</v>
       </c>
       <c r="D6" s="6">
         <f>SUM(B6:C6)</f>
-        <v>7666</v>
+        <v>7396</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1003,14 +1003,14 @@
         <v>39</v>
       </c>
       <c r="B7" s="6">
-        <v>3657</v>
+        <v>3604</v>
       </c>
       <c r="C7" s="6">
-        <v>3574</v>
+        <v>3734</v>
       </c>
       <c r="D7" s="6">
         <f>SUM(B7:C7)</f>
-        <v>7231</v>
+        <v>7338</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1018,14 +1018,14 @@
         <v>40</v>
       </c>
       <c r="B8" s="6">
-        <v>3538</v>
+        <v>3489</v>
       </c>
       <c r="C8" s="6">
-        <v>4054</v>
+        <v>4116</v>
       </c>
       <c r="D8" s="6">
         <f>SUM(B8:C8)</f>
-        <v>7592</v>
+        <v>7605</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1033,14 +1033,14 @@
         <v>41</v>
       </c>
       <c r="B9" s="6">
-        <v>3595</v>
+        <v>3637</v>
       </c>
       <c r="C9" s="6">
-        <v>4077</v>
+        <v>3993</v>
       </c>
       <c r="D9" s="6">
         <f>SUM(B9:C9)</f>
-        <v>7672</v>
+        <v>7630</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PAUSED (task169): portal round 4 repair in progress, the days out of custody filed and three ask devices cut
Methodology 4.1 now files that a member of the 2027 cohort is out of Department
custody from release until a return (SF21, judge 2's calendar basis). Ask devices:
legacy cases heard again after a rescission, parallel-run recommitments that reached
only the legacy system, carried-over detainers re-issued at go-live. The call and
every file it reads that no device touches are unchanged; the full build's gates
are running.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task169/golden/returns_projection_2027.xlsx
+++ b/task169/golden/returns_projection_2027.xlsx
@@ -76,7 +76,7 @@
     <t>A return is an ADM movement from the day after release to day 730 (methodology 3.1). Under the Act the Board recommits no one, so every return is a new court commitment.</t>
   </si>
   <si>
-    <t>Arrests per day out of Department custody in the first 730 days after each 2019 to September 2024 release to parole, by time since release, age, prior commitments, offence, sex and district.</t>
+    <t>Arrests per day out of Department custody in the first 730 days after each 2019 to September 2024 release to parole, by time since release, age, prior commitments, offence, sex and district, carried over all 730 days, the cohort being out of Department custody until a return (methodology 4.1).</t>
   </si>
   <si>
     <t>Each arrest's chance of a Department sentence and the time from arrest to admission are the courts' own, by charge grade (felony A-B, felony C-E, misdemeanour), from arrests to 30 June 2024 that went to court; arrests the Board answered by revoking parole are left out because no court decided them.</t>
@@ -88,7 +88,7 @@
     <t>Recommitments the Board ordered, 1 July 2025 to 30 June 2026, not rescinded by 30 June 2026</t>
   </si>
   <si>
-    <t>One recommitment per parolee per hearing: two reports taken up at one hearing are one order. Legacy system to 2 January 2026, new case system from 5 January.</t>
+    <t>One recommitment per parolee per hearing: two reports taken up at one hearing are one order, and a case heard again after a rescission keeps its later order. Legacy system to 2 January 2026 with the parallel-run decisions the new case system never received; new case system from 5 January.</t>
   </si>
   <si>
     <t>District office</t>
@@ -109,7 +109,7 @@
     <t>Parolee-days held on Board detainers in each district's county jails, 2025</t>
   </si>
   <si>
-    <t>A parolee held on two detainers at once is held once. Counting the day a detainer was lodged and not the day the person left; a legacy detainer with no lift date ended at the person's admission.</t>
+    <t>A parolee held on two detainers at once is held once. Counting the day a detainer was lodged and not the day the person left; a legacy detainer with no lift date ended at the person's admission; a carried-over detainer counted from its legacy lodge date, not the 5 January 2026 re-issue.</t>
   </si>
   <si>
     <t>January to June</t>
@@ -751,14 +751,14 @@
         <v>8</v>
       </c>
       <c r="C5" s="6">
-        <v>1277</v>
+        <v>1280</v>
       </c>
       <c r="D5" s="6">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E5" s="6">
         <f>C5+D5</f>
-        <v>1538</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -769,14 +769,14 @@
         <v>10</v>
       </c>
       <c r="C6" s="6">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="D6" s="6">
         <v>210</v>
       </c>
       <c r="E6" s="6">
         <f>C6+D6</f>
-        <v>831</v>
+        <v>832</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -787,14 +787,14 @@
         <v>12</v>
       </c>
       <c r="C7" s="6">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D7" s="6">
         <v>172</v>
       </c>
       <c r="E7" s="6">
         <f>C7+D7</f>
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -805,14 +805,14 @@
         <v>14</v>
       </c>
       <c r="C8" s="6">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D8" s="6">
         <v>149</v>
       </c>
       <c r="E8" s="6">
         <f>C8+D8</f>
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -821,15 +821,15 @@
       </c>
       <c r="C9" s="8">
         <f>SUM(C5:C8)</f>
-        <v>2382</v>
+        <v>2388</v>
       </c>
       <c r="D9" s="8">
         <f>SUM(D5:D8)</f>
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E9" s="8">
         <f>SUM(E5:E8)</f>
-        <v>3174</v>
+        <v>3181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>